<commit_message>
Add live invitation links to guest list
</commit_message>
<xml_diff>
--- a/outputs/wedding-rsvp/lista-de-invitados.xlsx
+++ b/outputs/wedding-rsvp/lista-de-invitados.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Invitados" sheetId="1" r:id="R406205f210f44488"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Invitados" sheetId="1" r:id="R0d981cbf893a448f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -127,7 +127,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="33">
+  <x:cellXfs count="35">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -175,6 +175,12 @@
     <x:xf numFmtId="0" fontId="4" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
     <x:xf numFmtId="200" fontId="4" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
@@ -194,10 +200,10 @@
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="5" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
+      <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="5" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
+      <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -405,7 +411,7 @@
     <x:col min="2" max="2" width="23" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="23" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="20" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="54" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="42" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="34" customHeight="1">
@@ -419,7 +425,7 @@
     </x:row>
     <x:row r="2" ht="34" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>Vista previa: estos enlaces solo funcionan en tu computadora por ahora. No los envíes todavía.</x:v>
+        <x:v>Enlaces oficiales: copia y envía solamente el enlace de la familia o persona correspondiente.</x:v>
       </x:c>
       <x:c r="B2" s="7"/>
       <x:c r="C2" s="7"/>
@@ -443,235 +449,235 @@
         <x:v>Enlace de invitación</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="25" customHeight="1">
+    <x:row r="5" ht="34" customHeight="1">
       <x:c r="A5" s="23" t="str">
         <x:v>Familia Palacios García</x:v>
       </x:c>
-      <x:c r="B5" s="27" t="n">
+      <x:c r="B5" s="29" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="C5" s="27" t="n">
+      <x:c r="C5" s="29" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="D5" s="29" t="str">
+      <x:c r="D5" s="31" t="str">
         <x:v>Familia</x:v>
       </x:c>
-      <x:c r="E5" s="31" t="str">
-        <x:v>http://127.0.0.1:4180/invite/DEMO1234#rsvp</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" ht="25" customHeight="1">
+      <x:c r="E5" s="33" t="str">
+        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/DEMO1234#rsvp</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="34" customHeight="1">
       <x:c r="A6" s="24" t="str">
         <x:v>McKay Stacey</x:v>
       </x:c>
-      <x:c r="B6" s="28" t="n">
+      <x:c r="B6" s="30" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="C6" s="28" t="n">
+      <x:c r="C6" s="30" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="D6" s="30" t="str">
+      <x:c r="D6" s="32" t="str">
         <x:v>Personal</x:v>
       </x:c>
-      <x:c r="E6" s="32" t="str">
-        <x:v>http://127.0.0.1:4180/invite/STACEY123#rsvp</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="25" customHeight="1">
+      <x:c r="E6" s="34" t="str">
+        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/STACEY123#rsvp</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="34" customHeight="1">
       <x:c r="A7" s="24" t="str"/>
-      <x:c r="B7" s="28"/>
-      <x:c r="C7" s="28"/>
-      <x:c r="D7" s="30" t="str"/>
-      <x:c r="E7" s="32" t="str"/>
-    </x:row>
-    <x:row r="8" ht="25" customHeight="1">
+      <x:c r="B7" s="30"/>
+      <x:c r="C7" s="30"/>
+      <x:c r="D7" s="32" t="str"/>
+      <x:c r="E7" s="34" t="str"/>
+    </x:row>
+    <x:row r="8" ht="34" customHeight="1">
       <x:c r="A8" s="24" t="str"/>
-      <x:c r="B8" s="28"/>
-      <x:c r="C8" s="28"/>
-      <x:c r="D8" s="30" t="str"/>
-      <x:c r="E8" s="32" t="str"/>
-    </x:row>
-    <x:row r="9" ht="25" customHeight="1">
+      <x:c r="B8" s="30"/>
+      <x:c r="C8" s="30"/>
+      <x:c r="D8" s="32" t="str"/>
+      <x:c r="E8" s="34" t="str"/>
+    </x:row>
+    <x:row r="9" ht="34" customHeight="1">
       <x:c r="A9" s="24" t="str"/>
-      <x:c r="B9" s="28"/>
-      <x:c r="C9" s="28"/>
-      <x:c r="D9" s="30" t="str"/>
-      <x:c r="E9" s="32" t="str"/>
-    </x:row>
-    <x:row r="10" ht="25" customHeight="1">
+      <x:c r="B9" s="30"/>
+      <x:c r="C9" s="30"/>
+      <x:c r="D9" s="32" t="str"/>
+      <x:c r="E9" s="34" t="str"/>
+    </x:row>
+    <x:row r="10" ht="34" customHeight="1">
       <x:c r="A10" s="24" t="str"/>
-      <x:c r="B10" s="28"/>
-      <x:c r="C10" s="28"/>
-      <x:c r="D10" s="30" t="str"/>
-      <x:c r="E10" s="32" t="str"/>
-    </x:row>
-    <x:row r="11" ht="25" customHeight="1">
+      <x:c r="B10" s="30"/>
+      <x:c r="C10" s="30"/>
+      <x:c r="D10" s="32" t="str"/>
+      <x:c r="E10" s="34" t="str"/>
+    </x:row>
+    <x:row r="11" ht="34" customHeight="1">
       <x:c r="A11" s="24" t="str"/>
-      <x:c r="B11" s="28"/>
-      <x:c r="C11" s="28"/>
-      <x:c r="D11" s="30" t="str"/>
-      <x:c r="E11" s="32" t="str"/>
-    </x:row>
-    <x:row r="12" ht="25" customHeight="1">
+      <x:c r="B11" s="30"/>
+      <x:c r="C11" s="30"/>
+      <x:c r="D11" s="32" t="str"/>
+      <x:c r="E11" s="34" t="str"/>
+    </x:row>
+    <x:row r="12" ht="34" customHeight="1">
       <x:c r="A12" s="24" t="str"/>
-      <x:c r="B12" s="28"/>
-      <x:c r="C12" s="28"/>
-      <x:c r="D12" s="30" t="str"/>
-      <x:c r="E12" s="32" t="str"/>
-    </x:row>
-    <x:row r="13" ht="25" customHeight="1">
+      <x:c r="B12" s="30"/>
+      <x:c r="C12" s="30"/>
+      <x:c r="D12" s="32" t="str"/>
+      <x:c r="E12" s="34" t="str"/>
+    </x:row>
+    <x:row r="13" ht="34" customHeight="1">
       <x:c r="A13" s="24" t="str"/>
-      <x:c r="B13" s="28"/>
-      <x:c r="C13" s="28"/>
-      <x:c r="D13" s="30" t="str"/>
-      <x:c r="E13" s="32" t="str"/>
-    </x:row>
-    <x:row r="14" ht="25" customHeight="1">
+      <x:c r="B13" s="30"/>
+      <x:c r="C13" s="30"/>
+      <x:c r="D13" s="32" t="str"/>
+      <x:c r="E13" s="34" t="str"/>
+    </x:row>
+    <x:row r="14" ht="34" customHeight="1">
       <x:c r="A14" s="24" t="str"/>
-      <x:c r="B14" s="28"/>
-      <x:c r="C14" s="28"/>
-      <x:c r="D14" s="30" t="str"/>
-      <x:c r="E14" s="32" t="str"/>
-    </x:row>
-    <x:row r="15" ht="25" customHeight="1">
+      <x:c r="B14" s="30"/>
+      <x:c r="C14" s="30"/>
+      <x:c r="D14" s="32" t="str"/>
+      <x:c r="E14" s="34" t="str"/>
+    </x:row>
+    <x:row r="15" ht="34" customHeight="1">
       <x:c r="A15" s="24" t="str"/>
-      <x:c r="B15" s="28"/>
-      <x:c r="C15" s="28"/>
-      <x:c r="D15" s="30" t="str"/>
-      <x:c r="E15" s="32" t="str"/>
-    </x:row>
-    <x:row r="16" ht="25" customHeight="1">
+      <x:c r="B15" s="30"/>
+      <x:c r="C15" s="30"/>
+      <x:c r="D15" s="32" t="str"/>
+      <x:c r="E15" s="34" t="str"/>
+    </x:row>
+    <x:row r="16" ht="34" customHeight="1">
       <x:c r="A16" s="24" t="str"/>
-      <x:c r="B16" s="28"/>
-      <x:c r="C16" s="28"/>
-      <x:c r="D16" s="30" t="str"/>
-      <x:c r="E16" s="32" t="str"/>
-    </x:row>
-    <x:row r="17" ht="25" customHeight="1">
+      <x:c r="B16" s="30"/>
+      <x:c r="C16" s="30"/>
+      <x:c r="D16" s="32" t="str"/>
+      <x:c r="E16" s="34" t="str"/>
+    </x:row>
+    <x:row r="17" ht="34" customHeight="1">
       <x:c r="A17" s="24" t="str"/>
-      <x:c r="B17" s="28"/>
-      <x:c r="C17" s="28"/>
-      <x:c r="D17" s="30" t="str"/>
-      <x:c r="E17" s="32" t="str"/>
-    </x:row>
-    <x:row r="18" ht="25" customHeight="1">
+      <x:c r="B17" s="30"/>
+      <x:c r="C17" s="30"/>
+      <x:c r="D17" s="32" t="str"/>
+      <x:c r="E17" s="34" t="str"/>
+    </x:row>
+    <x:row r="18" ht="34" customHeight="1">
       <x:c r="A18" s="24" t="str"/>
-      <x:c r="B18" s="28"/>
-      <x:c r="C18" s="28"/>
-      <x:c r="D18" s="30" t="str"/>
-      <x:c r="E18" s="32" t="str"/>
-    </x:row>
-    <x:row r="19" ht="25" customHeight="1">
+      <x:c r="B18" s="30"/>
+      <x:c r="C18" s="30"/>
+      <x:c r="D18" s="32" t="str"/>
+      <x:c r="E18" s="34" t="str"/>
+    </x:row>
+    <x:row r="19" ht="34" customHeight="1">
       <x:c r="A19" s="24" t="str"/>
-      <x:c r="B19" s="28"/>
-      <x:c r="C19" s="28"/>
-      <x:c r="D19" s="30" t="str"/>
-      <x:c r="E19" s="32" t="str"/>
-    </x:row>
-    <x:row r="20" ht="25" customHeight="1">
+      <x:c r="B19" s="30"/>
+      <x:c r="C19" s="30"/>
+      <x:c r="D19" s="32" t="str"/>
+      <x:c r="E19" s="34" t="str"/>
+    </x:row>
+    <x:row r="20" ht="34" customHeight="1">
       <x:c r="A20" s="24" t="str"/>
-      <x:c r="B20" s="28"/>
-      <x:c r="C20" s="28"/>
-      <x:c r="D20" s="30" t="str"/>
-      <x:c r="E20" s="32" t="str"/>
-    </x:row>
-    <x:row r="21" ht="25" customHeight="1">
+      <x:c r="B20" s="30"/>
+      <x:c r="C20" s="30"/>
+      <x:c r="D20" s="32" t="str"/>
+      <x:c r="E20" s="34" t="str"/>
+    </x:row>
+    <x:row r="21" ht="34" customHeight="1">
       <x:c r="A21" s="24" t="str"/>
-      <x:c r="B21" s="28"/>
-      <x:c r="C21" s="28"/>
-      <x:c r="D21" s="30" t="str"/>
-      <x:c r="E21" s="32" t="str"/>
-    </x:row>
-    <x:row r="22" ht="25" customHeight="1">
+      <x:c r="B21" s="30"/>
+      <x:c r="C21" s="30"/>
+      <x:c r="D21" s="32" t="str"/>
+      <x:c r="E21" s="34" t="str"/>
+    </x:row>
+    <x:row r="22" ht="34" customHeight="1">
       <x:c r="A22" s="24" t="str"/>
-      <x:c r="B22" s="28"/>
-      <x:c r="C22" s="28"/>
-      <x:c r="D22" s="30" t="str"/>
-      <x:c r="E22" s="32" t="str"/>
-    </x:row>
-    <x:row r="23" ht="25" customHeight="1">
+      <x:c r="B22" s="30"/>
+      <x:c r="C22" s="30"/>
+      <x:c r="D22" s="32" t="str"/>
+      <x:c r="E22" s="34" t="str"/>
+    </x:row>
+    <x:row r="23" ht="34" customHeight="1">
       <x:c r="A23" s="24" t="str"/>
-      <x:c r="B23" s="28"/>
-      <x:c r="C23" s="28"/>
-      <x:c r="D23" s="30" t="str"/>
-      <x:c r="E23" s="32" t="str"/>
-    </x:row>
-    <x:row r="24" ht="25" customHeight="1">
+      <x:c r="B23" s="30"/>
+      <x:c r="C23" s="30"/>
+      <x:c r="D23" s="32" t="str"/>
+      <x:c r="E23" s="34" t="str"/>
+    </x:row>
+    <x:row r="24" ht="34" customHeight="1">
       <x:c r="A24" s="24" t="str"/>
-      <x:c r="B24" s="28"/>
-      <x:c r="C24" s="28"/>
-      <x:c r="D24" s="30" t="str"/>
-      <x:c r="E24" s="32" t="str"/>
-    </x:row>
-    <x:row r="25" ht="25" customHeight="1">
+      <x:c r="B24" s="30"/>
+      <x:c r="C24" s="30"/>
+      <x:c r="D24" s="32" t="str"/>
+      <x:c r="E24" s="34" t="str"/>
+    </x:row>
+    <x:row r="25" ht="34" customHeight="1">
       <x:c r="A25" s="24" t="str"/>
-      <x:c r="B25" s="28"/>
-      <x:c r="C25" s="28"/>
-      <x:c r="D25" s="30" t="str"/>
-      <x:c r="E25" s="32" t="str"/>
-    </x:row>
-    <x:row r="26" ht="25" customHeight="1">
+      <x:c r="B25" s="30"/>
+      <x:c r="C25" s="30"/>
+      <x:c r="D25" s="32" t="str"/>
+      <x:c r="E25" s="34" t="str"/>
+    </x:row>
+    <x:row r="26" ht="34" customHeight="1">
       <x:c r="A26" s="24" t="str"/>
-      <x:c r="B26" s="28"/>
-      <x:c r="C26" s="28"/>
-      <x:c r="D26" s="30" t="str"/>
-      <x:c r="E26" s="32" t="str"/>
-    </x:row>
-    <x:row r="27" ht="25" customHeight="1">
+      <x:c r="B26" s="30"/>
+      <x:c r="C26" s="30"/>
+      <x:c r="D26" s="32" t="str"/>
+      <x:c r="E26" s="34" t="str"/>
+    </x:row>
+    <x:row r="27" ht="34" customHeight="1">
       <x:c r="A27" s="24" t="str"/>
-      <x:c r="B27" s="28"/>
-      <x:c r="C27" s="28"/>
-      <x:c r="D27" s="30" t="str"/>
-      <x:c r="E27" s="32" t="str"/>
-    </x:row>
-    <x:row r="28" ht="25" customHeight="1">
+      <x:c r="B27" s="30"/>
+      <x:c r="C27" s="30"/>
+      <x:c r="D27" s="32" t="str"/>
+      <x:c r="E27" s="34" t="str"/>
+    </x:row>
+    <x:row r="28" ht="34" customHeight="1">
       <x:c r="A28" s="24" t="str"/>
-      <x:c r="B28" s="28"/>
-      <x:c r="C28" s="28"/>
-      <x:c r="D28" s="30" t="str"/>
-      <x:c r="E28" s="32" t="str"/>
-    </x:row>
-    <x:row r="29" ht="25" customHeight="1">
+      <x:c r="B28" s="30"/>
+      <x:c r="C28" s="30"/>
+      <x:c r="D28" s="32" t="str"/>
+      <x:c r="E28" s="34" t="str"/>
+    </x:row>
+    <x:row r="29" ht="34" customHeight="1">
       <x:c r="A29" s="24" t="str"/>
-      <x:c r="B29" s="28"/>
-      <x:c r="C29" s="28"/>
-      <x:c r="D29" s="30" t="str"/>
-      <x:c r="E29" s="32" t="str"/>
-    </x:row>
-    <x:row r="30" ht="25" customHeight="1">
+      <x:c r="B29" s="30"/>
+      <x:c r="C29" s="30"/>
+      <x:c r="D29" s="32" t="str"/>
+      <x:c r="E29" s="34" t="str"/>
+    </x:row>
+    <x:row r="30" ht="34" customHeight="1">
       <x:c r="A30" s="24" t="str"/>
-      <x:c r="B30" s="28"/>
-      <x:c r="C30" s="28"/>
-      <x:c r="D30" s="30" t="str"/>
-      <x:c r="E30" s="32" t="str"/>
-    </x:row>
-    <x:row r="31" ht="25" customHeight="1">
+      <x:c r="B30" s="30"/>
+      <x:c r="C30" s="30"/>
+      <x:c r="D30" s="32" t="str"/>
+      <x:c r="E30" s="34" t="str"/>
+    </x:row>
+    <x:row r="31" ht="34" customHeight="1">
       <x:c r="A31" s="24" t="str"/>
-      <x:c r="B31" s="28"/>
-      <x:c r="C31" s="28"/>
-      <x:c r="D31" s="30" t="str"/>
-      <x:c r="E31" s="32" t="str"/>
-    </x:row>
-    <x:row r="32" ht="25" customHeight="1">
+      <x:c r="B31" s="30"/>
+      <x:c r="C31" s="30"/>
+      <x:c r="D31" s="32" t="str"/>
+      <x:c r="E31" s="34" t="str"/>
+    </x:row>
+    <x:row r="32" ht="34" customHeight="1">
       <x:c r="A32" s="24" t="str"/>
-      <x:c r="B32" s="28"/>
-      <x:c r="C32" s="28"/>
-      <x:c r="D32" s="30" t="str"/>
-      <x:c r="E32" s="32" t="str"/>
-    </x:row>
-    <x:row r="33" ht="25" customHeight="1">
+      <x:c r="B32" s="30"/>
+      <x:c r="C32" s="30"/>
+      <x:c r="D32" s="32" t="str"/>
+      <x:c r="E32" s="34" t="str"/>
+    </x:row>
+    <x:row r="33" ht="34" customHeight="1">
       <x:c r="A33" s="24" t="str"/>
-      <x:c r="B33" s="28"/>
-      <x:c r="C33" s="28"/>
-      <x:c r="D33" s="30" t="str"/>
-      <x:c r="E33" s="32" t="str"/>
-    </x:row>
-    <x:row r="34" ht="25" customHeight="1">
+      <x:c r="B33" s="30"/>
+      <x:c r="C33" s="30"/>
+      <x:c r="D33" s="32" t="str"/>
+      <x:c r="E33" s="34" t="str"/>
+    </x:row>
+    <x:row r="34" ht="34" customHeight="1">
       <x:c r="A34" s="24" t="str"/>
-      <x:c r="B34" s="28"/>
-      <x:c r="C34" s="28"/>
-      <x:c r="D34" s="30" t="str"/>
-      <x:c r="E34" s="32" t="str"/>
+      <x:c r="B34" s="30"/>
+      <x:c r="C34" s="30"/>
+      <x:c r="D34" s="32" t="str"/>
+      <x:c r="E34" s="34" t="str"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>

<commit_message>
Fix invitation assets and sync updated guest list
</commit_message>
<xml_diff>
--- a/outputs/wedding-rsvp/lista-de-invitados.xlsx
+++ b/outputs/wedding-rsvp/lista-de-invitados.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Invitados" sheetId="1" r:id="R89ea0798cdea463c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Invitados" sheetId="1" r:id="R43ec0abb25bd41b5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -95,6 +95,9 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Familia Palacios Mercado</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Magdalena &amp; Daniel</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -895,11 +898,21 @@
       <x:c r="E28" s="11"/>
     </x:row>
     <x:row r="29" ht="34" customHeight="1">
-      <x:c r="A29" s="5"/>
-      <x:c r="B29" s="7"/>
-      <x:c r="C29" s="7"/>
-      <x:c r="D29" s="9"/>
-      <x:c r="E29" s="11"/>
+      <x:c r="A29" s="5" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="B29" s="7">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C29" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D29" s="9" t="str">
+        <x:v>Pareja</x:v>
+      </x:c>
+      <x:c r="E29" s="11" t="str">
+        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/B25BF43BF3DF#rsvp</x:v>
+      </x:c>
     </x:row>
     <x:row r="30" ht="34" customHeight="1">
       <x:c r="A30" s="5"/>

</xml_diff>

<commit_message>
Sync expanded guest list and simplify couple invites
</commit_message>
<xml_diff>
--- a/outputs/wedding-rsvp/lista-de-invitados.xlsx
+++ b/outputs/wedding-rsvp/lista-de-invitados.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Invitados" sheetId="1" r:id="R43ec0abb25bd41b5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Invitados" sheetId="1" r:id="R3fb665d64ad743f7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -99,12 +99,84 @@
   <x:si>
     <x:t xml:space="preserve">Magdalena &amp; Daniel</x:t>
   </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Familia Medina</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Familia Leon</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Eber &amp; Emma</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Norma &amp; Wendy</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Fanny &amp; Angela</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Familia de Ericka</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Ana &amp; Roge</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Fredy &amp; Rosy</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Marisol &amp; Juan Carlos</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Lau</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Jacky</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Faby</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Pau</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Paty &amp; Juan Carlos</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Arturo &amp; Gracia</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Katy &amp; Kevin</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Familia de Naty</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Diana &amp; Esposo</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Francisca</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Familia de Anel</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Familia de Eliza</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Familia de Mia</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Familia Niño</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Tere &amp; Novio</x:t>
+  </x:si>
 </x:sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="6">
+  <x:fonts count="9">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -137,8 +209,23 @@
       <x:color rgb="FF2F6F73"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color theme="10"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF786250"/>
+      <x:name val="Aptos"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF3F7E88"/>
+      <x:name val="Aptos"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="6">
+  <x:fills count="7">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -165,8 +252,13 @@
         <x:fgColor rgb="FFFFFEFC"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFDFC"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="6">
+  <x:borders count="9">
     <x:border/>
     <x:border>
       <x:left style="thin">
@@ -211,11 +303,33 @@
         <x:color rgb="FFE7D6C3"/>
       </x:bottom>
     </x:border>
+    <x:border>
+      <x:bottom style="thin">
+        <x:color rgb="FFE8D8C8"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:top style="thin">
+        <x:color rgb="FFE8D8C8"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFE8D8C8"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:top style="thin">
+        <x:color rgb="FFE8D8C8"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFE7D6C3"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
-  <x:cellStyleXfs count="1">
+  <x:cellStyleXfs count="2">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="14">
+  <x:cellXfs count="61">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
@@ -244,20 +358,154 @@
     <x:xf numFmtId="0" fontId="4" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
-    </x:xf>
     <x:xf numFmtId="0" fontId="5" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="1" fontId="4" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="5" borderId="5" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="5" borderId="4" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="1" fontId="4" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="1" fontId="4" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="1" fontId="4" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="1" fontId="7" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="1" fontId="7" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="1" fontId="7" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="6" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="1" fontId="7" fillId="6" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="6" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="6" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="6" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="1" fontId="7" fillId="6" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="6" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="6" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="6" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="6" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="1" fontId="7" fillId="6" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="6" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="6" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="6" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="6" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="6" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="6" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="6" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
   </x:cellXfs>
-  <x:cellStyles count="1">
+  <x:cellStyles count="2">
+    <x:cellStyle name="Hyperlink" xfId="1"/>
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
 </x:styleSheet>
@@ -458,29 +706,31 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <x:cols>
-    <x:col min="1" max="1" width="38" customWidth="1"/>
-    <x:col min="2" max="3" width="23" customWidth="1"/>
-    <x:col min="4" max="4" width="20" customWidth="1"/>
-    <x:col min="5" max="5" width="42" customWidth="1"/>
+    <x:col min="1" max="1" width="28" hidden="0" customWidth="1"/>
+    <x:col min="2" max="3" width="15.6640625" customWidth="1"/>
+    <x:col min="4" max="4" width="19" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="48" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="18" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="34" customHeight="1">
-      <x:c r="A1" s="12" t="s">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="B1" s="12"/>
-      <x:c r="C1" s="12"/>
-      <x:c r="D1" s="12"/>
-      <x:c r="E1" s="12"/>
+      <x:c r="A1" s="16" t="s">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="B1" s="16"/>
+      <x:c r="C1" s="16"/>
+      <x:c r="D1" s="16"/>
+      <x:c r="E1" s="16"/>
     </x:row>
     <x:row r="2" ht="34" customHeight="1">
-      <x:c r="A2" s="13" t="str">
+      <x:c r="A2" s="17" t="str">
         <x:v>Enlaces oficiales: copia y envía solamente el enlace de la familia, pareja o persona correspondiente.</x:v>
       </x:c>
-      <x:c r="B2" s="13"/>
-      <x:c r="C2" s="13"/>
-      <x:c r="D2" s="13"/>
-      <x:c r="E2" s="13"/>
+      <x:c r="B2" s="17"/>
+      <x:c r="C2" s="17"/>
+      <x:c r="D2" s="17"/>
+      <x:c r="E2" s="17"/>
     </x:row>
     <x:row r="4" ht="32" customHeight="1">
       <x:c r="A4" s="1" t="s">
@@ -500,454 +750,847 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="4" t="s">
+      <x:c r="A5" s="46" t="s">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="B5" s="6">
+      <x:c r="B5" s="44">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="C5" s="6" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="D5" s="8" t="str">
-        <x:v>Familia</x:v>
-      </x:c>
-      <x:c r="E5" s="10" t="str">
+      <x:c r="C5" s="44" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D5" s="45" t="str">
+        <x:v>Familia</x:v>
+      </x:c>
+      <x:c r="E5" s="57" t="str">
         <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/DEMO1234#rsvp</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="34" customHeight="1">
-      <x:c r="A6" s="5" t="s">
+      <x:c r="A6" s="50" t="s">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="B6" s="7">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C6" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="D6" s="9" t="str">
+      <x:c r="B6" s="48">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C6" s="48" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D6" s="49" t="str">
         <x:v>Individual</x:v>
       </x:c>
-      <x:c r="E6" s="11" t="str">
+      <x:c r="E6" s="58" t="str">
         <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/STACEY123#rsvp</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="34" customHeight="1">
-      <x:c r="A7" s="5" t="s">
+      <x:c r="A7" s="50" t="s">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="B7" s="7">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C7" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="D7" s="9" t="str">
+      <x:c r="B7" s="48">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C7" s="48" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D7" s="49" t="str">
         <x:v>Individual</x:v>
       </x:c>
-      <x:c r="E7" s="11" t="str">
+      <x:c r="E7" s="58" t="str">
         <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/0F6F1F34F89B#rsvp</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="34" customHeight="1">
-      <x:c r="A8" s="5" t="s">
+      <x:c r="A8" s="50" t="s">
         <x:v>9</x:v>
       </x:c>
-      <x:c r="B8" s="7">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C8" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="D8" s="9" t="str">
+      <x:c r="B8" s="48">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C8" s="48" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D8" s="49" t="str">
         <x:v>Individual</x:v>
       </x:c>
-      <x:c r="E8" s="11" t="str">
+      <x:c r="E8" s="58" t="str">
         <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/ACF0340BED3B#rsvp</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="34" customHeight="1">
-      <x:c r="A9" s="5" t="s">
+      <x:c r="A9" s="50" t="s">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="B9" s="7">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C9" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="D9" s="9" t="str">
+      <x:c r="B9" s="48">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C9" s="48" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D9" s="49" t="str">
         <x:v>Individual</x:v>
       </x:c>
-      <x:c r="E9" s="11" t="str">
+      <x:c r="E9" s="58" t="str">
         <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/5E1FC4622B8E#rsvp</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="34" customHeight="1">
-      <x:c r="A10" s="5" t="s">
+      <x:c r="A10" s="50" t="s">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="B10" s="7">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C10" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="D10" s="9" t="str">
+      <x:c r="B10" s="48">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C10" s="48" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D10" s="49" t="str">
         <x:v>Individual</x:v>
       </x:c>
-      <x:c r="E10" s="11" t="str">
+      <x:c r="E10" s="58" t="str">
         <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/80CD79B61F2C#rsvp</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="34" customHeight="1">
-      <x:c r="A11" s="5" t="s">
+      <x:c r="A11" s="50" t="s">
         <x:v>12</x:v>
       </x:c>
-      <x:c r="B11" s="7">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C11" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="D11" s="9" t="str">
+      <x:c r="B11" s="48">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C11" s="48" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D11" s="49" t="str">
         <x:v>Individual</x:v>
       </x:c>
-      <x:c r="E11" s="11" t="str">
+      <x:c r="E11" s="58" t="str">
         <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/8B629E341F49#rsvp</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="34" customHeight="1">
-      <x:c r="A12" s="5" t="s">
+      <x:c r="A12" s="50" t="s">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="B12" s="7">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="C12" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="D12" s="9" t="str">
+      <x:c r="B12" s="48">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C12" s="48" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D12" s="49" t="str">
         <x:v>Pareja</x:v>
       </x:c>
-      <x:c r="E12" s="11" t="str">
+      <x:c r="E12" s="58" t="str">
         <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/04B5EBC43DF9#rsvp</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="34" customHeight="1">
-      <x:c r="A13" s="5" t="s">
+      <x:c r="A13" s="50" t="s">
         <x:v>14</x:v>
       </x:c>
-      <x:c r="B13" s="7">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C13" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="D13" s="9" t="str">
+      <x:c r="B13" s="48">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C13" s="48" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D13" s="49" t="str">
         <x:v>Individual</x:v>
       </x:c>
-      <x:c r="E13" s="11" t="str">
+      <x:c r="E13" s="58" t="str">
         <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/267615B915A9#rsvp</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="34" customHeight="1">
-      <x:c r="A14" s="5" t="s">
+      <x:c r="A14" s="50" t="s">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="B14" s="7">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C14" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="D14" s="9" t="str">
+      <x:c r="B14" s="48">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C14" s="48" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D14" s="49" t="str">
         <x:v>Individual</x:v>
       </x:c>
-      <x:c r="E14" s="11" t="str">
+      <x:c r="E14" s="58" t="str">
         <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/5C31C44AA8FF#rsvp</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="34" customHeight="1">
-      <x:c r="A15" s="5" t="s">
+      <x:c r="A15" s="50" t="s">
         <x:v>16</x:v>
       </x:c>
-      <x:c r="B15" s="7">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C15" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="D15" s="9" t="str">
+      <x:c r="B15" s="48">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C15" s="48" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D15" s="49" t="str">
         <x:v>Individual</x:v>
       </x:c>
-      <x:c r="E15" s="11" t="str">
+      <x:c r="E15" s="58" t="str">
         <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/777B6D895849#rsvp</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="34" customHeight="1">
-      <x:c r="A16" s="5" t="s">
+      <x:c r="A16" s="50" t="s">
         <x:v>17</x:v>
       </x:c>
-      <x:c r="B16" s="7">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="C16" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="D16" s="9" t="str">
+      <x:c r="B16" s="48">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C16" s="48" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D16" s="49" t="str">
         <x:v>Pareja</x:v>
       </x:c>
-      <x:c r="E16" s="11" t="str">
+      <x:c r="E16" s="58" t="str">
         <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/DD7FBF881F11#rsvp</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="34" customHeight="1">
-      <x:c r="A17" s="5" t="s">
+      <x:c r="A17" s="50" t="s">
         <x:v>18</x:v>
       </x:c>
-      <x:c r="B17" s="7">
+      <x:c r="B17" s="48">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="C17" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="D17" s="9" t="str">
-        <x:v>Familia</x:v>
-      </x:c>
-      <x:c r="E17" s="11" t="str">
+      <x:c r="C17" s="48" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D17" s="49" t="str">
+        <x:v>Familia</x:v>
+      </x:c>
+      <x:c r="E17" s="58" t="str">
         <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/EF8690606661#rsvp</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="34" customHeight="1">
-      <x:c r="A18" s="5" t="s">
+      <x:c r="A18" s="50" t="s">
         <x:v>19</x:v>
       </x:c>
-      <x:c r="B18" s="7">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="C18" s="7" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="D18" s="9" t="str">
-        <x:v>Familia</x:v>
-      </x:c>
-      <x:c r="E18" s="11" t="str">
+      <x:c r="B18" s="48">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C18" s="48" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D18" s="49" t="str">
+        <x:v>Familia</x:v>
+      </x:c>
+      <x:c r="E18" s="58" t="str">
         <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/A70F1BE059EA#rsvp</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="34" customHeight="1">
-      <x:c r="A19" s="5" t="s">
+      <x:c r="A19" s="50" t="s">
         <x:v>20</x:v>
       </x:c>
-      <x:c r="B19" s="7">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="C19" s="7" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="D19" s="9" t="str">
-        <x:v>Familia</x:v>
-      </x:c>
-      <x:c r="E19" s="11" t="str">
+      <x:c r="B19" s="48">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C19" s="48" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D19" s="49" t="str">
+        <x:v>Familia</x:v>
+      </x:c>
+      <x:c r="E19" s="58" t="str">
         <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/734446FDCC1C#rsvp</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="34" customHeight="1">
-      <x:c r="A20" s="5" t="s">
+      <x:c r="A20" s="50" t="s">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="B20" s="7">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C20" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="D20" s="9" t="str">
+      <x:c r="B20" s="48">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C20" s="48" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D20" s="49" t="str">
         <x:v>Individual</x:v>
       </x:c>
-      <x:c r="E20" s="11" t="str">
+      <x:c r="E20" s="58" t="str">
         <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/BA0DC53A08D6#rsvp</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="34" customHeight="1">
-      <x:c r="A21" s="5" t="s">
+      <x:c r="A21" s="50" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="B21" s="7">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C21" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="D21" s="9" t="str">
+      <x:c r="B21" s="48">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C21" s="48" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D21" s="49" t="str">
         <x:v>Individual</x:v>
       </x:c>
-      <x:c r="E21" s="11" t="str">
+      <x:c r="E21" s="58" t="str">
         <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/E008B1CDC1DA#rsvp</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="34" customHeight="1">
-      <x:c r="A22" s="5" t="s">
+      <x:c r="A22" s="50" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="B22" s="7">
+      <x:c r="B22" s="48">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="C22" s="7" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="D22" s="9" t="str">
-        <x:v>Familia</x:v>
-      </x:c>
-      <x:c r="E22" s="11" t="str">
+      <x:c r="C22" s="48" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D22" s="49" t="str">
+        <x:v>Familia</x:v>
+      </x:c>
+      <x:c r="E22" s="58" t="str">
         <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/4F69964650FA#rsvp</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="34" customHeight="1">
-      <x:c r="A23" s="5" t="s">
+      <x:c r="A23" s="50" t="s">
         <x:v>24</x:v>
       </x:c>
-      <x:c r="B23" s="7">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C23" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="D23" s="9" t="str">
+      <x:c r="B23" s="48">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C23" s="48" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D23" s="49" t="str">
         <x:v>Individual</x:v>
       </x:c>
-      <x:c r="E23" s="11" t="str">
+      <x:c r="E23" s="58" t="str">
         <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/2B449C292516#rsvp</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="34" customHeight="1">
-      <x:c r="A24" s="5" t="s">
+      <x:c r="A24" s="50" t="s">
         <x:v>25</x:v>
       </x:c>
-      <x:c r="B24" s="7">
+      <x:c r="B24" s="48">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="C24" s="7" t="n">
+      <x:c r="C24" s="48" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="D24" s="9" t="str">
-        <x:v>Familia</x:v>
-      </x:c>
-      <x:c r="E24" s="11" t="str">
+      <x:c r="D24" s="49" t="str">
+        <x:v>Familia</x:v>
+      </x:c>
+      <x:c r="E24" s="58" t="str">
         <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/83773353FC78#rsvp</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="34" customHeight="1">
-      <x:c r="A25" s="5" t="s">
+      <x:c r="A25" s="50" t="s">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="B25" s="7">
+      <x:c r="B25" s="48">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="C25" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="D25" s="9" t="str">
-        <x:v>Familia</x:v>
-      </x:c>
-      <x:c r="E25" s="11" t="str">
+      <x:c r="C25" s="48" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D25" s="49" t="str">
+        <x:v>Familia</x:v>
+      </x:c>
+      <x:c r="E25" s="58" t="str">
         <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/8AFDD077D4C0#rsvp</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="34" customHeight="1">
-      <x:c r="A26" s="5" t="s">
+      <x:c r="A26" s="50" t="s">
         <x:v>27</x:v>
       </x:c>
-      <x:c r="B26" s="7">
+      <x:c r="B26" s="48">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="C26" s="7" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="D26" s="9" t="str">
-        <x:v>Familia</x:v>
-      </x:c>
-      <x:c r="E26" s="11" t="str">
+      <x:c r="C26" s="48" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D26" s="49" t="str">
+        <x:v>Familia</x:v>
+      </x:c>
+      <x:c r="E26" s="58" t="str">
         <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/4F121B878BB1#rsvp</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="34" customHeight="1">
-      <x:c r="A27" s="5" t="s">
+      <x:c r="A27" s="50" t="s">
         <x:v>28</x:v>
       </x:c>
-      <x:c r="B27" s="7">
+      <x:c r="B27" s="48">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="C27" s="7" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="D27" s="9" t="str">
-        <x:v>Familia</x:v>
-      </x:c>
-      <x:c r="E27" s="11" t="str">
+      <x:c r="C27" s="48" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D27" s="49" t="str">
+        <x:v>Familia</x:v>
+      </x:c>
+      <x:c r="E27" s="58" t="str">
         <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/0189765496A9#rsvp</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="34" customHeight="1">
-      <x:c r="A28" s="5"/>
-      <x:c r="B28" s="7"/>
-      <x:c r="C28" s="7"/>
-      <x:c r="D28" s="9"/>
-      <x:c r="E28" s="11"/>
+      <x:c r="A28" s="50"/>
+      <x:c r="B28" s="48"/>
+      <x:c r="C28" s="48"/>
+      <x:c r="D28" s="49"/>
+      <x:c r="E28" s="58"/>
     </x:row>
     <x:row r="29" ht="34" customHeight="1">
-      <x:c r="A29" s="5" t="s">
+      <x:c r="A29" s="50" t="s">
         <x:v>29</x:v>
       </x:c>
-      <x:c r="B29" s="7">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="C29" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="D29" s="9" t="str">
+      <x:c r="B29" s="48">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C29" s="48" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D29" s="49" t="str">
         <x:v>Pareja</x:v>
       </x:c>
-      <x:c r="E29" s="11" t="str">
+      <x:c r="E29" s="58" t="str">
         <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/B25BF43BF3DF#rsvp</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="34" customHeight="1">
-      <x:c r="A30" s="5"/>
-      <x:c r="B30" s="7"/>
-      <x:c r="C30" s="7"/>
-      <x:c r="D30" s="9"/>
-      <x:c r="E30" s="11"/>
+      <x:c r="A30" s="50" t="s">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="B30" s="48">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C30" s="48" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D30" s="49" t="str">
+        <x:v>Familia</x:v>
+      </x:c>
+      <x:c r="E30" s="58" t="str">
+        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/80B16A4F86AD#rsvp</x:v>
+      </x:c>
     </x:row>
     <x:row r="31" ht="34" customHeight="1">
-      <x:c r="A31" s="5"/>
-      <x:c r="B31" s="7"/>
-      <x:c r="C31" s="7"/>
-      <x:c r="D31" s="9"/>
-      <x:c r="E31" s="11"/>
+      <x:c r="A31" s="50" t="s">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="B31" s="48">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="C31" s="48" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D31" s="49" t="str">
+        <x:v>Familia</x:v>
+      </x:c>
+      <x:c r="E31" s="58" t="str">
+        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/B77E4BCCBA73#rsvp</x:v>
+      </x:c>
     </x:row>
     <x:row r="32" ht="34" customHeight="1">
-      <x:c r="A32" s="5"/>
-      <x:c r="B32" s="7"/>
-      <x:c r="C32" s="7"/>
-      <x:c r="D32" s="9"/>
-      <x:c r="E32" s="11"/>
+      <x:c r="A32" s="50" t="s">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="B32" s="48">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C32" s="48" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D32" s="49" t="str">
+        <x:v>Familia</x:v>
+      </x:c>
+      <x:c r="E32" s="58" t="str">
+        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/12EB6141467A#rsvp</x:v>
+      </x:c>
     </x:row>
     <x:row r="33" ht="34" customHeight="1">
-      <x:c r="A33" s="5"/>
-      <x:c r="B33" s="7"/>
-      <x:c r="C33" s="7"/>
-      <x:c r="D33" s="9"/>
-      <x:c r="E33" s="11"/>
+      <x:c r="A33" s="50" t="s">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="B33" s="48">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C33" s="48" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D33" s="49" t="str">
+        <x:v>Familia</x:v>
+      </x:c>
+      <x:c r="E33" s="58" t="str">
+        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/769CC28AE31E#rsvp</x:v>
+      </x:c>
     </x:row>
     <x:row r="34" ht="34" customHeight="1">
-      <x:c r="A34" s="5"/>
-      <x:c r="B34" s="7"/>
-      <x:c r="C34" s="7"/>
-      <x:c r="D34" s="9"/>
-      <x:c r="E34" s="11"/>
+      <x:c r="A34" s="50" t="s">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="B34" s="48">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C34" s="48" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D34" s="49" t="str">
+        <x:v>Familia</x:v>
+      </x:c>
+      <x:c r="E34" s="58" t="str">
+        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/68371C8C4E81#rsvp</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="34" customHeight="1">
+      <x:c r="A35" s="50" t="s">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="B35" s="48">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C35" s="49" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D35" s="49" t="str">
+        <x:v>Familia</x:v>
+      </x:c>
+      <x:c r="E35" s="58" t="str">
+        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/368FE148DB63#rsvp</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" ht="34" customHeight="1">
+      <x:c r="A36" s="50" t="s">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="B36" s="48">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C36" s="49" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D36" s="49" t="str">
+        <x:v>Pareja</x:v>
+      </x:c>
+      <x:c r="E36" s="58" t="str">
+        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/9903175B9BE6#rsvp</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="34" customHeight="1">
+      <x:c r="A37" s="50" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="B37" s="48">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C37" s="49" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D37" s="49" t="str">
+        <x:v>Pareja</x:v>
+      </x:c>
+      <x:c r="E37" s="58" t="str">
+        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/BE1FE04982F2#rsvp</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="34" customHeight="1">
+      <x:c r="A38" s="50" t="s">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="B38" s="48">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C38" s="49" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D38" s="49" t="str">
+        <x:v>Familia</x:v>
+      </x:c>
+      <x:c r="E38" s="58" t="str">
+        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/0FAC4F0C43C1#rsvp</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" ht="34" customHeight="1">
+      <x:c r="A39" s="50" t="s">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="B39" s="48">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C39" s="49" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D39" s="49" t="str">
+        <x:v>Familia</x:v>
+      </x:c>
+      <x:c r="E39" s="58" t="str">
+        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/8BAB060F25DE#rsvp</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="34" customHeight="1">
+      <x:c r="A40" s="50" t="s">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="B40" s="48">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C40" s="49" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D40" s="49" t="str">
+        <x:v>Individual</x:v>
+      </x:c>
+      <x:c r="E40" s="58" t="str">
+        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/867E04448417#rsvp</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41" ht="34" customHeight="1">
+      <x:c r="A41" s="50" t="s">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="B41" s="48">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C41" s="49" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D41" s="49" t="str">
+        <x:v>Individual</x:v>
+      </x:c>
+      <x:c r="E41" s="58" t="str">
+        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/3281BF87522B#rsvp</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42" ht="34" customHeight="1">
+      <x:c r="A42" s="50" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="B42" s="48">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C42" s="49" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D42" s="49" t="str">
+        <x:v>Individual</x:v>
+      </x:c>
+      <x:c r="E42" s="58" t="str">
+        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/643D092E0777#rsvp</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43" ht="34" customHeight="1">
+      <x:c r="A43" s="50" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="B43" s="48">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C43" s="49" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D43" s="49" t="str">
+        <x:v>Pareja</x:v>
+      </x:c>
+      <x:c r="E43" s="58" t="str">
+        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/32874971241C#rsvp</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44" ht="34" customHeight="1">
+      <x:c r="A44" s="50" t="s">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="B44" s="48">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C44" s="49" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D44" s="49" t="str">
+        <x:v>Familia</x:v>
+      </x:c>
+      <x:c r="E44" s="58" t="str">
+        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/407A9534932A#rsvp</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" ht="34" customHeight="1">
+      <x:c r="A45" s="50" t="s">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="B45" s="48">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C45" s="49" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D45" s="49" t="str">
+        <x:v>Pareja</x:v>
+      </x:c>
+      <x:c r="E45" s="58" t="str">
+        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/A0B09870FB51#rsvp</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46" ht="34" customHeight="1">
+      <x:c r="A46" s="50" t="s">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="B46" s="48">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C46" s="49" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D46" s="49" t="str">
+        <x:v>Pareja</x:v>
+      </x:c>
+      <x:c r="E46" s="58" t="str">
+        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/36F03F13C250#rsvp</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47" ht="34" customHeight="1">
+      <x:c r="A47" s="50" t="s">
+        <x:v>46</x:v>
+      </x:c>
+      <x:c r="B47" s="48">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C47" s="49" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D47" s="49" t="str">
+        <x:v>Familia</x:v>
+      </x:c>
+      <x:c r="E47" s="58" t="str">
+        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/FB5CE2FD53FB#rsvp</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48" ht="34" customHeight="1">
+      <x:c r="A48" s="50" t="s">
+        <x:v>47</x:v>
+      </x:c>
+      <x:c r="B48" s="48">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C48" s="49" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D48" s="49" t="str">
+        <x:v>Pareja</x:v>
+      </x:c>
+      <x:c r="E48" s="58" t="str">
+        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/45BA4CCD5593#rsvp</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49" ht="34" customHeight="1">
+      <x:c r="A49" s="50" t="s">
+        <x:v>48</x:v>
+      </x:c>
+      <x:c r="B49" s="48">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C49" s="49" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D49" s="49" t="str">
+        <x:v>Individual</x:v>
+      </x:c>
+      <x:c r="E49" s="58" t="str">
+        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/CB697F934939#rsvp</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50" ht="34" customHeight="1">
+      <x:c r="A50" s="50" t="s">
+        <x:v>49</x:v>
+      </x:c>
+      <x:c r="B50" s="48">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C50" s="49" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D50" s="49" t="str">
+        <x:v>Familia</x:v>
+      </x:c>
+      <x:c r="E50" s="58" t="str">
+        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/717064338477#rsvp</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51" ht="34" customHeight="1">
+      <x:c r="A51" s="50" t="s">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="B51" s="48">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C51" s="49" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D51" s="49" t="str">
+        <x:v>Familia</x:v>
+      </x:c>
+      <x:c r="E51" s="58" t="str">
+        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/E81581A736C3#rsvp</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52" ht="34" customHeight="1">
+      <x:c r="A52" s="50" t="s">
+        <x:v>51</x:v>
+      </x:c>
+      <x:c r="B52" s="48">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C52" s="49" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D52" s="49" t="str">
+        <x:v>Familia</x:v>
+      </x:c>
+      <x:c r="E52" s="58" t="str">
+        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/386436E97AF2#rsvp</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53" ht="34" customHeight="1">
+      <x:c r="A53" s="50" t="s">
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="B53" s="48">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C53" s="49" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D53" s="49" t="str">
+        <x:v>Familia</x:v>
+      </x:c>
+      <x:c r="E53" s="58" t="str">
+        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/5A4DD3F9F8AA#rsvp</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54" ht="34" customHeight="1">
+      <x:c r="A54" s="56" t="s">
+        <x:v>53</x:v>
+      </x:c>
+      <x:c r="B54" s="53">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C54" s="54" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D54" s="54" t="str">
+        <x:v>Familia</x:v>
+      </x:c>
+      <x:c r="E54" s="58" t="str">
+        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/6EC9E29F0C61#rsvp</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55">
+      <x:c r="C55" s="13"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -966,6 +1609,11 @@
       <x:formula1>"Individual,Pareja,Familia"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
+  <x:hyperlinks>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="Rd5198fc3117349be"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="Rbd4fa18b640e4411"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="R72ec2a78caeb4b4c"/>
+  </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Fix gallery slide alignment and mark bride family
</commit_message>
<xml_diff>
--- a/outputs/wedding-rsvp/lista-de-invitados.xlsx
+++ b/outputs/wedding-rsvp/lista-de-invitados.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Invitados" sheetId="1" r:id="R3fb665d64ad743f7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Invitados" sheetId="1" r:id="R857e6da12ef54ed9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -176,7 +176,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="9">
+  <x:fonts count="10">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -224,8 +224,14 @@
       <x:color rgb="FF3F7E88"/>
       <x:name val="Aptos"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Aptos"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="7">
+  <x:fills count="8">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -257,8 +263,13 @@
         <x:fgColor rgb="FFFFFDFC"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF737A48"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="9">
+  <x:borders count="10">
     <x:border/>
     <x:border>
       <x:left style="thin">
@@ -324,12 +335,20 @@
         <x:color rgb="FFE7D6C3"/>
       </x:bottom>
     </x:border>
+    <x:border>
+      <x:top style="medium">
+        <x:color rgb="FF5A6038"/>
+      </x:top>
+      <x:bottom style="medium">
+        <x:color rgb="FF5A6038"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="2">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="61">
+  <x:cellXfs count="72">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
@@ -502,6 +521,39 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="8" fillId="6" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="7" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="1" fontId="7" fillId="7" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="7" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="7" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="7" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="1" fontId="9" fillId="7" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="7" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="7" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="1" fontId="9" fillId="7" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="7" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="7" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="2">
@@ -1140,12 +1192,22 @@
         <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/0189765496A9#rsvp</x:v>
       </x:c>
     </x:row>
-    <x:row r="28" ht="34" customHeight="1">
-      <x:c r="A28" s="50"/>
-      <x:c r="B28" s="48"/>
-      <x:c r="C28" s="48"/>
-      <x:c r="D28" s="49"/>
-      <x:c r="E28" s="58"/>
+    <x:row r="28" ht="30" customHeight="1">
+      <x:c r="A28" s="71" t="str">
+        <x:v>FAMILIA DE LA NOVIA</x:v>
+      </x:c>
+      <x:c r="B28" s="69" t="str">
+        <x:v>FAMILIA DE LA NOVIA</x:v>
+      </x:c>
+      <x:c r="C28" s="69" t="str">
+        <x:v>FAMILIA DE LA NOVIA</x:v>
+      </x:c>
+      <x:c r="D28" s="70" t="str">
+        <x:v>FAMILIA DE LA NOVIA</x:v>
+      </x:c>
+      <x:c r="E28" s="71" t="str">
+        <x:v>FAMILIA DE LA NOVIA</x:v>
+      </x:c>
     </x:row>
     <x:row r="29" ht="34" customHeight="1">
       <x:c r="A29" s="50" t="s">
@@ -1596,6 +1658,7 @@
   <x:mergeCells>
     <x:mergeCell ref="A1:E1"/>
     <x:mergeCell ref="A2:E2"/>
+    <x:mergeCell ref="A28:E28"/>
   </x:mergeCells>
   <x:dataValidations count="3">
     <x:dataValidation type="whole" sqref="B5:C34">
@@ -1610,9 +1673,9 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="Rd5198fc3117349be"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="Rbd4fa18b640e4411"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="R72ec2a78caeb4b4c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="Rd6e5ce11a4e04cf4"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="R63dcdca92aab4665"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="R2a513d6b203b4289"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Add bride family gift preferences and top-opening links
</commit_message>
<xml_diff>
--- a/outputs/wedding-rsvp/lista-de-invitados.xlsx
+++ b/outputs/wedding-rsvp/lista-de-invitados.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Invitados" sheetId="1" r:id="R857e6da12ef54ed9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Invitados" sheetId="1" r:id="Rb1fe4863141c4e3f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -231,7 +231,7 @@
       <x:name val="Aptos"/>
     </x:font>
   </x:fonts>
-  <x:fills count="8">
+  <x:fills count="9">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -261,6 +261,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFFFDFC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF737A48"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -348,7 +353,7 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="72">
+  <x:cellXfs count="75">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
@@ -554,6 +559,15 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="9" fillId="7" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="8" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="1" fontId="9" fillId="8" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="8" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="2">
@@ -815,7 +829,7 @@
         <x:v>Familia</x:v>
       </x:c>
       <x:c r="E5" s="57" t="str">
-        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/DEMO1234#rsvp</x:v>
+        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/DEMO1234</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="34" customHeight="1">
@@ -832,7 +846,7 @@
         <x:v>Individual</x:v>
       </x:c>
       <x:c r="E6" s="58" t="str">
-        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/STACEY123#rsvp</x:v>
+        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/STACEY123</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="34" customHeight="1">
@@ -849,7 +863,7 @@
         <x:v>Individual</x:v>
       </x:c>
       <x:c r="E7" s="58" t="str">
-        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/0F6F1F34F89B#rsvp</x:v>
+        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/0F6F1F34F89B</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="34" customHeight="1">
@@ -866,7 +880,7 @@
         <x:v>Individual</x:v>
       </x:c>
       <x:c r="E8" s="58" t="str">
-        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/ACF0340BED3B#rsvp</x:v>
+        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/ACF0340BED3B</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="34" customHeight="1">
@@ -883,7 +897,7 @@
         <x:v>Individual</x:v>
       </x:c>
       <x:c r="E9" s="58" t="str">
-        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/5E1FC4622B8E#rsvp</x:v>
+        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/5E1FC4622B8E</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="34" customHeight="1">
@@ -900,7 +914,7 @@
         <x:v>Individual</x:v>
       </x:c>
       <x:c r="E10" s="58" t="str">
-        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/80CD79B61F2C#rsvp</x:v>
+        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/80CD79B61F2C</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="34" customHeight="1">
@@ -917,7 +931,7 @@
         <x:v>Individual</x:v>
       </x:c>
       <x:c r="E11" s="58" t="str">
-        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/8B629E341F49#rsvp</x:v>
+        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/8B629E341F49</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="34" customHeight="1">
@@ -934,7 +948,7 @@
         <x:v>Pareja</x:v>
       </x:c>
       <x:c r="E12" s="58" t="str">
-        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/04B5EBC43DF9#rsvp</x:v>
+        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/04B5EBC43DF9</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="34" customHeight="1">
@@ -951,7 +965,7 @@
         <x:v>Individual</x:v>
       </x:c>
       <x:c r="E13" s="58" t="str">
-        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/267615B915A9#rsvp</x:v>
+        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/267615B915A9</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="34" customHeight="1">
@@ -968,7 +982,7 @@
         <x:v>Individual</x:v>
       </x:c>
       <x:c r="E14" s="58" t="str">
-        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/5C31C44AA8FF#rsvp</x:v>
+        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/5C31C44AA8FF</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="34" customHeight="1">
@@ -985,7 +999,7 @@
         <x:v>Individual</x:v>
       </x:c>
       <x:c r="E15" s="58" t="str">
-        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/777B6D895849#rsvp</x:v>
+        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/777B6D895849</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="34" customHeight="1">
@@ -1002,7 +1016,7 @@
         <x:v>Pareja</x:v>
       </x:c>
       <x:c r="E16" s="58" t="str">
-        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/DD7FBF881F11#rsvp</x:v>
+        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/DD7FBF881F11</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="34" customHeight="1">
@@ -1019,7 +1033,7 @@
         <x:v>Familia</x:v>
       </x:c>
       <x:c r="E17" s="58" t="str">
-        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/EF8690606661#rsvp</x:v>
+        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/EF8690606661</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="34" customHeight="1">
@@ -1036,7 +1050,7 @@
         <x:v>Familia</x:v>
       </x:c>
       <x:c r="E18" s="58" t="str">
-        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/A70F1BE059EA#rsvp</x:v>
+        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/A70F1BE059EA</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="34" customHeight="1">
@@ -1053,7 +1067,7 @@
         <x:v>Familia</x:v>
       </x:c>
       <x:c r="E19" s="58" t="str">
-        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/734446FDCC1C#rsvp</x:v>
+        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/734446FDCC1C</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="34" customHeight="1">
@@ -1070,7 +1084,7 @@
         <x:v>Individual</x:v>
       </x:c>
       <x:c r="E20" s="58" t="str">
-        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/BA0DC53A08D6#rsvp</x:v>
+        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/BA0DC53A08D6</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="34" customHeight="1">
@@ -1087,7 +1101,7 @@
         <x:v>Individual</x:v>
       </x:c>
       <x:c r="E21" s="58" t="str">
-        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/E008B1CDC1DA#rsvp</x:v>
+        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/E008B1CDC1DA</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="34" customHeight="1">
@@ -1104,7 +1118,7 @@
         <x:v>Familia</x:v>
       </x:c>
       <x:c r="E22" s="58" t="str">
-        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/4F69964650FA#rsvp</x:v>
+        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/4F69964650FA</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="34" customHeight="1">
@@ -1121,7 +1135,7 @@
         <x:v>Individual</x:v>
       </x:c>
       <x:c r="E23" s="58" t="str">
-        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/2B449C292516#rsvp</x:v>
+        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/2B449C292516</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="34" customHeight="1">
@@ -1138,7 +1152,7 @@
         <x:v>Familia</x:v>
       </x:c>
       <x:c r="E24" s="58" t="str">
-        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/83773353FC78#rsvp</x:v>
+        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/83773353FC78</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="34" customHeight="1">
@@ -1155,7 +1169,7 @@
         <x:v>Familia</x:v>
       </x:c>
       <x:c r="E25" s="58" t="str">
-        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/8AFDD077D4C0#rsvp</x:v>
+        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/8AFDD077D4C0</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="34" customHeight="1">
@@ -1172,7 +1186,7 @@
         <x:v>Familia</x:v>
       </x:c>
       <x:c r="E26" s="58" t="str">
-        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/4F121B878BB1#rsvp</x:v>
+        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/4F121B878BB1</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="34" customHeight="1">
@@ -1189,23 +1203,23 @@
         <x:v>Familia</x:v>
       </x:c>
       <x:c r="E27" s="58" t="str">
-        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/0189765496A9#rsvp</x:v>
+        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/0189765496A9</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="30" customHeight="1">
-      <x:c r="A28" s="71" t="str">
+      <x:c r="A28" s="72" t="str">
         <x:v>FAMILIA DE LA NOVIA</x:v>
       </x:c>
-      <x:c r="B28" s="69" t="str">
+      <x:c r="B28" s="73" t="str">
         <x:v>FAMILIA DE LA NOVIA</x:v>
       </x:c>
-      <x:c r="C28" s="69" t="str">
+      <x:c r="C28" s="73" t="str">
         <x:v>FAMILIA DE LA NOVIA</x:v>
       </x:c>
-      <x:c r="D28" s="70" t="str">
+      <x:c r="D28" s="74" t="str">
         <x:v>FAMILIA DE LA NOVIA</x:v>
       </x:c>
-      <x:c r="E28" s="71" t="str">
+      <x:c r="E28" s="72" t="str">
         <x:v>FAMILIA DE LA NOVIA</x:v>
       </x:c>
     </x:row>
@@ -1223,7 +1237,7 @@
         <x:v>Pareja</x:v>
       </x:c>
       <x:c r="E29" s="58" t="str">
-        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/B25BF43BF3DF#rsvp</x:v>
+        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/B25BF43BF3DF</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="34" customHeight="1">
@@ -1240,7 +1254,7 @@
         <x:v>Familia</x:v>
       </x:c>
       <x:c r="E30" s="58" t="str">
-        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/80B16A4F86AD#rsvp</x:v>
+        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/80B16A4F86AD</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="34" customHeight="1">
@@ -1257,7 +1271,7 @@
         <x:v>Familia</x:v>
       </x:c>
       <x:c r="E31" s="58" t="str">
-        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/B77E4BCCBA73#rsvp</x:v>
+        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/B77E4BCCBA73</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="34" customHeight="1">
@@ -1274,7 +1288,7 @@
         <x:v>Familia</x:v>
       </x:c>
       <x:c r="E32" s="58" t="str">
-        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/12EB6141467A#rsvp</x:v>
+        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/12EB6141467A</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="34" customHeight="1">
@@ -1291,7 +1305,7 @@
         <x:v>Familia</x:v>
       </x:c>
       <x:c r="E33" s="58" t="str">
-        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/769CC28AE31E#rsvp</x:v>
+        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/769CC28AE31E</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="34" customHeight="1">
@@ -1308,7 +1322,7 @@
         <x:v>Familia</x:v>
       </x:c>
       <x:c r="E34" s="58" t="str">
-        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/68371C8C4E81#rsvp</x:v>
+        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/68371C8C4E81</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="34" customHeight="1">
@@ -1325,7 +1339,7 @@
         <x:v>Familia</x:v>
       </x:c>
       <x:c r="E35" s="58" t="str">
-        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/368FE148DB63#rsvp</x:v>
+        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/368FE148DB63</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="34" customHeight="1">
@@ -1342,7 +1356,7 @@
         <x:v>Pareja</x:v>
       </x:c>
       <x:c r="E36" s="58" t="str">
-        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/9903175B9BE6#rsvp</x:v>
+        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/9903175B9BE6</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="34" customHeight="1">
@@ -1359,7 +1373,7 @@
         <x:v>Pareja</x:v>
       </x:c>
       <x:c r="E37" s="58" t="str">
-        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/BE1FE04982F2#rsvp</x:v>
+        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/BE1FE04982F2</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="34" customHeight="1">
@@ -1376,7 +1390,7 @@
         <x:v>Familia</x:v>
       </x:c>
       <x:c r="E38" s="58" t="str">
-        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/0FAC4F0C43C1#rsvp</x:v>
+        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/0FAC4F0C43C1</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="34" customHeight="1">
@@ -1393,7 +1407,7 @@
         <x:v>Familia</x:v>
       </x:c>
       <x:c r="E39" s="58" t="str">
-        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/8BAB060F25DE#rsvp</x:v>
+        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/8BAB060F25DE</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="34" customHeight="1">
@@ -1410,7 +1424,7 @@
         <x:v>Individual</x:v>
       </x:c>
       <x:c r="E40" s="58" t="str">
-        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/867E04448417#rsvp</x:v>
+        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/867E04448417</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="34" customHeight="1">
@@ -1427,7 +1441,7 @@
         <x:v>Individual</x:v>
       </x:c>
       <x:c r="E41" s="58" t="str">
-        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/3281BF87522B#rsvp</x:v>
+        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/3281BF87522B</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="34" customHeight="1">
@@ -1444,7 +1458,7 @@
         <x:v>Individual</x:v>
       </x:c>
       <x:c r="E42" s="58" t="str">
-        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/643D092E0777#rsvp</x:v>
+        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/643D092E0777</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="34" customHeight="1">
@@ -1461,7 +1475,7 @@
         <x:v>Pareja</x:v>
       </x:c>
       <x:c r="E43" s="58" t="str">
-        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/32874971241C#rsvp</x:v>
+        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/32874971241C</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="34" customHeight="1">
@@ -1478,7 +1492,7 @@
         <x:v>Familia</x:v>
       </x:c>
       <x:c r="E44" s="58" t="str">
-        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/407A9534932A#rsvp</x:v>
+        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/407A9534932A</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="34" customHeight="1">
@@ -1495,7 +1509,7 @@
         <x:v>Pareja</x:v>
       </x:c>
       <x:c r="E45" s="58" t="str">
-        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/A0B09870FB51#rsvp</x:v>
+        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/A0B09870FB51</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="34" customHeight="1">
@@ -1512,7 +1526,7 @@
         <x:v>Pareja</x:v>
       </x:c>
       <x:c r="E46" s="58" t="str">
-        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/36F03F13C250#rsvp</x:v>
+        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/36F03F13C250</x:v>
       </x:c>
     </x:row>
     <x:row r="47" ht="34" customHeight="1">
@@ -1529,7 +1543,7 @@
         <x:v>Familia</x:v>
       </x:c>
       <x:c r="E47" s="58" t="str">
-        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/FB5CE2FD53FB#rsvp</x:v>
+        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/FB5CE2FD53FB</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="34" customHeight="1">
@@ -1546,7 +1560,7 @@
         <x:v>Pareja</x:v>
       </x:c>
       <x:c r="E48" s="58" t="str">
-        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/45BA4CCD5593#rsvp</x:v>
+        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/45BA4CCD5593</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="34" customHeight="1">
@@ -1563,7 +1577,7 @@
         <x:v>Individual</x:v>
       </x:c>
       <x:c r="E49" s="58" t="str">
-        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/CB697F934939#rsvp</x:v>
+        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/CB697F934939</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="34" customHeight="1">
@@ -1580,7 +1594,7 @@
         <x:v>Familia</x:v>
       </x:c>
       <x:c r="E50" s="58" t="str">
-        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/717064338477#rsvp</x:v>
+        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/717064338477</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="34" customHeight="1">
@@ -1597,7 +1611,7 @@
         <x:v>Familia</x:v>
       </x:c>
       <x:c r="E51" s="58" t="str">
-        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/E81581A736C3#rsvp</x:v>
+        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/E81581A736C3</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="34" customHeight="1">
@@ -1614,7 +1628,7 @@
         <x:v>Familia</x:v>
       </x:c>
       <x:c r="E52" s="58" t="str">
-        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/386436E97AF2#rsvp</x:v>
+        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/386436E97AF2</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="34" customHeight="1">
@@ -1631,7 +1645,7 @@
         <x:v>Familia</x:v>
       </x:c>
       <x:c r="E53" s="58" t="str">
-        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/5A4DD3F9F8AA#rsvp</x:v>
+        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/5A4DD3F9F8AA</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="34" customHeight="1">
@@ -1648,7 +1662,7 @@
         <x:v>Familia</x:v>
       </x:c>
       <x:c r="E54" s="58" t="str">
-        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/6EC9E29F0C61#rsvp</x:v>
+        <x:v>https://regnier-alizee-boda.joseregnier14.chatgpt.site/invite/6EC9E29F0C61</x:v>
       </x:c>
     </x:row>
     <x:row r="55">
@@ -1673,9 +1687,9 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="Rd6e5ce11a4e04cf4"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="R63dcdca92aab4665"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="R2a513d6b203b4289"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="Rea6ab7fc67084283"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="R1b0d3d9a71c444e9"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="R3ebf3d15bf6c45b4"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>